<commit_message>
Updated Case + BOM
</commit_message>
<xml_diff>
--- a/BOM/BOM.xlsx
+++ b/BOM/BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\marinboard\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4812F401-6AA1-4E5D-97FD-D8F74A33C3A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A742A81-FCCB-460F-82FB-CF35A654A948}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5803721C-F8C9-41F6-8A44-40A526ECC638}"/>
   </bookViews>
@@ -547,7 +547,7 @@
         <v>11</v>
       </c>
       <c r="C8" s="2">
-        <v>31.2</v>
+        <v>69.28</v>
       </c>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.25">
@@ -588,8 +588,8 @@
         <v>12</v>
       </c>
       <c r="C12">
-        <f>6.57+7.52+11.56+31.2+2.06+9.29+7.9</f>
-        <v>76.099999999999994</v>
+        <f>6.57+7.52+11.56+69.28+2.06+9.29+7.9</f>
+        <v>114.18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>